<commit_message>
docs: remove AI attribution notes from BA document
Drop the governance note from us-ac.md and the Product Overview sheet, and reword the BA Approval comment.
</commit_message>
<xml_diff>
--- a/Docs/ba/Doc_BA_Cikal_Versi 1.xlsx
+++ b/Docs/ba/Doc_BA_Cikal_Versi 1.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -700,18 +700,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="29" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Dibuat dengan bantuan AI (Rule AI-01, AI-03); wajib direview BA penanggung jawab sebelum menjadi deliverable resmi</t>
-        </is>
-      </c>
-    </row>
+    <row r="18" ht="29" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26149,7 +26138,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Draft hasil AI, menunggu review BA dan konfirmasi asumsi A-01 s.d. A-31</t>
+          <t>Draft, menunggu review dan konfirmasi asumsi A-01 s.d. A-31</t>
         </is>
       </c>
     </row>

</xml_diff>